<commit_message>
Adding bound on import of gas
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_SUP_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_SUP_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB09237A-E2EF-46ED-B2E1-52A47896CD68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7B98A8F-AB7A-4D54-8199-819CF61BFE8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="68">
   <si>
     <t>~FI_Process</t>
   </si>
@@ -208,9 +208,6 @@
     <t>winoff_potential</t>
   </si>
   <si>
-    <t>wnid offshore potential</t>
-  </si>
-  <si>
     <t>Electricity import from Finland</t>
   </si>
   <si>
@@ -254,6 +251,15 @@
   </si>
   <si>
     <t>windoff</t>
+  </si>
+  <si>
+    <t>wind offshore potential</t>
+  </si>
+  <si>
+    <t>ktoe</t>
+  </si>
+  <si>
+    <t>ACT_BND</t>
   </si>
 </sst>
 </file>
@@ -452,7 +458,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
@@ -492,6 +498,8 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="17">
     <cellStyle name="40% - Accent2 2" xfId="11" xr:uid="{087B65A6-0941-47D0-A448-C10B046F140C}"/>
@@ -805,7 +813,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C768FA58-8399-45BE-8875-71A71258D648}">
-  <dimension ref="B4:W27"/>
+  <dimension ref="B2:W27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
@@ -828,6 +836,22 @@
     <col min="22" max="22" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="2" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="K2" t="s">
+        <v>66</v>
+      </c>
+      <c r="L2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1.163E-2</v>
+      </c>
+    </row>
     <row r="4" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -862,7 +886,7 @@
         <v>14</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>15</v>
@@ -884,6 +908,9 @@
       </c>
       <c r="L5" s="14" t="s">
         <v>21</v>
+      </c>
+      <c r="M5" s="14" t="s">
+        <v>67</v>
       </c>
       <c r="P5" s="5" t="s">
         <v>1</v>
@@ -926,6 +953,7 @@
       <c r="J6" s="16"/>
       <c r="K6" s="16"/>
       <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
       <c r="P6" s="12" t="s">
         <v>28</v>
       </c>
@@ -986,7 +1014,7 @@
         <v>9</v>
       </c>
       <c r="R7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="S7" s="1" t="s">
         <v>6</v>
@@ -1030,7 +1058,7 @@
         <v>10</v>
       </c>
       <c r="R8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S8" s="1" t="s">
         <v>6</v>
@@ -1074,7 +1102,7 @@
         <v>12</v>
       </c>
       <c r="R9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="S9" s="1" t="s">
         <v>6</v>
@@ -1118,7 +1146,7 @@
         <v>11</v>
       </c>
       <c r="R10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S10" s="1" t="s">
         <v>6</v>
@@ -1135,7 +1163,7 @@
         <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G11" s="17">
         <v>97.330783938814534</v>
@@ -1158,7 +1186,7 @@
     </row>
     <row r="12" spans="2:23" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G12" s="17">
         <v>35.496509410102867</v>
@@ -1181,10 +1209,14 @@
     </row>
     <row r="13" spans="2:23" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G13" s="17">
         <v>46.935294117647068</v>
+      </c>
+      <c r="M13" s="20">
+        <f>90.7*L3</f>
+        <v>1.0548409999999999</v>
       </c>
       <c r="P13" s="1" t="s">
         <v>5</v>
@@ -1207,7 +1239,7 @@
         <v>41</v>
       </c>
       <c r="D14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G14" s="17">
         <v>0.36000000000000004</v>
@@ -1230,7 +1262,7 @@
     </row>
     <row r="15" spans="2:23" x14ac:dyDescent="0.25">
       <c r="D15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G15" s="17">
         <v>0.36000000000000004</v>
@@ -1253,7 +1285,7 @@
     </row>
     <row r="16" spans="2:23" x14ac:dyDescent="0.25">
       <c r="D16" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G16" s="17">
         <v>46.249920000000003</v>
@@ -1265,7 +1297,7 @@
         <v>49</v>
       </c>
       <c r="R16" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="S16" s="1" t="s">
         <v>6</v>
@@ -1274,45 +1306,48 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>43</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G17" s="17">
         <v>6</v>
       </c>
-    </row>
-    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="P17" s="19"/>
+      <c r="S17" s="19"/>
+      <c r="T17" s="19"/>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>45</v>
       </c>
       <c r="D18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G18">
         <v>0.36000000000000004</v>
       </c>
     </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G19">
         <v>0.36000000000000004</v>
       </c>
     </row>
-    <row r="20" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>49</v>
       </c>
       <c r="D20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G20">
         <v>0.36000000000000004</v>
@@ -1323,16 +1358,16 @@
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
     </row>
-    <row r="21" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="K21" s="1"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
       <c r="S21" s="8"/>
     </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
       <c r="K27" s="1"/>
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>

</xml_diff>

<commit_message>
Mistake ACT_BND for gas was accidetnally put to oil
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_SUP_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_SUP_v1.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7B98A8F-AB7A-4D54-8199-819CF61BFE8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA489383-9FC8-45C8-8E6C-1BFA581C2E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supply" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,6 +40,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={E038209F-90E0-4A15-8D63-AF2C49B09543}</author>
+    <author>tc={911363B4-7669-41CE-B552-D3EFD733FC50}</author>
   </authors>
   <commentList>
     <comment ref="D4" authorId="0" shapeId="0" xr:uid="{E038209F-90E0-4A15-8D63-AF2C49B09543}">
@@ -51,6 +53,14 @@
     refineries</t>
       </text>
     </comment>
+    <comment ref="I7" authorId="1" shapeId="0" xr:uid="{911363B4-7669-41CE-B552-D3EFD733FC50}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Can remove, no capacity variable</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -271,7 +281,7 @@
     <numFmt numFmtId="164" formatCode="\Te\x\t"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -342,6 +352,12 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="186"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -458,7 +474,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
@@ -498,7 +514,6 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="17">
@@ -808,6 +823,9 @@
   <threadedComment ref="D4" dT="2026-05-28T08:00:29.37" personId="{929FE2BB-984B-46A4-91E1-AB3A16D849D3}" id="{FE89220A-8A49-4561-8962-F3D0F49B38B4}" parentId="{E038209F-90E0-4A15-8D63-AF2C49B09543}">
     <text>refineries</text>
   </threadedComment>
+  <threadedComment ref="I7" dT="2026-06-11T10:48:10.54" personId="{929FE2BB-984B-46A4-91E1-AB3A16D849D3}" id="{911363B4-7669-41CE-B552-D3EFD733FC50}">
+    <text>Can remove, no capacity variable</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
@@ -1191,6 +1209,10 @@
       <c r="G12" s="17">
         <v>35.496509410102867</v>
       </c>
+      <c r="M12" s="19">
+        <f>90.7*L3</f>
+        <v>1.0548409999999999</v>
+      </c>
       <c r="P12" s="1" t="s">
         <v>5</v>
       </c>
@@ -1214,10 +1236,6 @@
       <c r="G13" s="17">
         <v>46.935294117647068</v>
       </c>
-      <c r="M13" s="20">
-        <f>90.7*L3</f>
-        <v>1.0548409999999999</v>
-      </c>
       <c r="P13" s="1" t="s">
         <v>5</v>
       </c>
@@ -1306,7 +1324,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>43</v>
       </c>
@@ -1316,11 +1334,8 @@
       <c r="G17" s="17">
         <v>6</v>
       </c>
-      <c r="P17" s="19"/>
-      <c r="S17" s="19"/>
-      <c r="T17" s="19"/>
-    </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>45</v>
       </c>
@@ -1331,7 +1346,7 @@
         <v>0.36000000000000004</v>
       </c>
     </row>
-    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>47</v>
       </c>
@@ -1342,7 +1357,7 @@
         <v>0.36000000000000004</v>
       </c>
     </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>49</v>
       </c>
@@ -1358,16 +1373,16 @@
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:19" x14ac:dyDescent="0.25">
       <c r="K21" s="1"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
       <c r="S21" s="8"/>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:19" x14ac:dyDescent="0.25">
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:19" x14ac:dyDescent="0.25">
       <c r="K27" s="1"/>
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>

</xml_diff>

<commit_message>
Removing act boundary on gas
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_SUP_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_SUP_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA489383-9FC8-45C8-8E6C-1BFA581C2E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7912F7E-3D75-4B25-9B2A-5F73C810E7FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1209,7 +1209,7 @@
       <c r="G12" s="17">
         <v>35.496509410102867</v>
       </c>
-      <c r="M12" s="19">
+      <c r="N12" s="19">
         <f>90.7*L3</f>
         <v>1.0548409999999999</v>
       </c>

</xml_diff>

<commit_message>
Removing "0" column if there is no attribute defined
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_SUP_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_SUP_v1.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7912F7E-3D75-4B25-9B2A-5F73C810E7FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21258C10-E4E6-498A-B8F8-F75A7FC777CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supply" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -53,7 +52,7 @@
     refineries</t>
       </text>
     </comment>
-    <comment ref="I7" authorId="1" shapeId="0" xr:uid="{911363B4-7669-41CE-B552-D3EFD733FC50}">
+    <comment ref="H7" authorId="1" shapeId="0" xr:uid="{911363B4-7669-41CE-B552-D3EFD733FC50}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -281,7 +280,7 @@
     <numFmt numFmtId="164" formatCode="\Te\x\t"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -352,12 +351,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="186"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -823,7 +816,7 @@
   <threadedComment ref="D4" dT="2026-05-28T08:00:29.37" personId="{929FE2BB-984B-46A4-91E1-AB3A16D849D3}" id="{FE89220A-8A49-4561-8962-F3D0F49B38B4}" parentId="{E038209F-90E0-4A15-8D63-AF2C49B09543}">
     <text>refineries</text>
   </threadedComment>
-  <threadedComment ref="I7" dT="2026-06-11T10:48:10.54" personId="{929FE2BB-984B-46A4-91E1-AB3A16D849D3}" id="{911363B4-7669-41CE-B552-D3EFD733FC50}">
+  <threadedComment ref="H7" dT="2026-06-11T10:48:10.54" personId="{929FE2BB-984B-46A4-91E1-AB3A16D849D3}" id="{911363B4-7669-41CE-B552-D3EFD733FC50}">
     <text>Can remove, no capacity variable</text>
   </threadedComment>
 </ThreadedComments>
@@ -831,46 +824,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C768FA58-8399-45BE-8875-71A71258D648}">
-  <dimension ref="B2:W27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:V27"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.453125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" customWidth="1"/>
-    <col min="8" max="8" width="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.42578125" customWidth="1"/>
-    <col min="10" max="10" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" customWidth="1"/>
-    <col min="12" max="14" width="14.140625" customWidth="1"/>
-    <col min="15" max="15" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="28.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.140625" customWidth="1"/>
+    <col min="5" max="5" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.1796875" customWidth="1"/>
+    <col min="7" max="7" width="9.453125" customWidth="1"/>
+    <col min="8" max="8" width="8.453125" customWidth="1"/>
+    <col min="9" max="9" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.7265625" customWidth="1"/>
+    <col min="11" max="13" width="14.1796875" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="K2" t="s">
+    <row r="1" spans="2:22" x14ac:dyDescent="0.35">
+      <c r="J1" t="s">
         <v>66</v>
       </c>
-      <c r="L2" t="s">
+      <c r="K1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="K3">
+    <row r="2" spans="2:22" x14ac:dyDescent="0.35">
+      <c r="J2">
         <v>1</v>
       </c>
-      <c r="L3">
+      <c r="K2">
         <v>1.163E-2</v>
       </c>
     </row>
-    <row r="4" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
       <c r="D4" s="11" t="s">
@@ -882,18 +874,17 @@
       <c r="H4" s="10"/>
       <c r="I4" s="10"/>
       <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="P4" s="4" t="s">
+      <c r="O4" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="Q4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-    </row>
-    <row r="5" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="13" t="s">
         <v>2</v>
       </c>
@@ -912,50 +903,47 @@
       <c r="G5" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="14">
-        <v>0</v>
+      <c r="H5" s="14" t="s">
+        <v>17</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="M5" s="14" t="s">
         <v>67</v>
       </c>
+      <c r="O5" s="5" t="s">
+        <v>1</v>
+      </c>
       <c r="P5" s="5" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="R5" s="5" t="s">
         <v>3</v>
       </c>
+      <c r="R5" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="S5" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="U5" s="6" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="V5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="W5" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="2:23" s="7" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:22" s="7" customFormat="1" ht="46.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B6" s="12" t="s">
         <v>36</v>
       </c>
@@ -967,37 +955,36 @@
         <v>37</v>
       </c>
       <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
+      <c r="I6" s="16"/>
       <c r="J6" s="16"/>
       <c r="K6" s="16"/>
       <c r="L6" s="16"/>
-      <c r="M6" s="16"/>
+      <c r="O6" s="12" t="s">
+        <v>28</v>
+      </c>
       <c r="P6" s="12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q6" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="R6" s="12" t="s">
         <v>30</v>
       </c>
+      <c r="R6" s="15" t="s">
+        <v>31</v>
+      </c>
       <c r="S6" s="15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T6" s="15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="U6" s="15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="V6" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="W6" s="15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>9</v>
       </c>
@@ -1011,40 +998,37 @@
         <v>40.49</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>1000</v>
       </c>
       <c r="I7">
-        <v>1000</v>
+        <v>50</v>
       </c>
       <c r="J7">
+        <v>1.016</v>
+      </c>
+      <c r="K7">
+        <v>0.8</v>
+      </c>
+      <c r="O7" t="s">
+        <v>5</v>
+      </c>
+      <c r="P7" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q7" t="s">
         <v>50</v>
       </c>
-      <c r="K7">
-        <v>1.016</v>
-      </c>
-      <c r="L7">
-        <v>0.8</v>
-      </c>
-      <c r="P7" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>9</v>
-      </c>
-      <c r="R7" t="s">
-        <v>50</v>
-      </c>
-      <c r="S7" s="1" t="s">
+      <c r="R7" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="S7" t="s">
+        <v>7</v>
+      </c>
       <c r="T7" t="s">
-        <v>7</v>
-      </c>
-      <c r="U7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>10</v>
       </c>
@@ -1058,37 +1042,34 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>3</v>
+        <v>1000</v>
       </c>
       <c r="I8">
-        <v>1000</v>
+        <v>50</v>
       </c>
       <c r="J8">
-        <v>50</v>
-      </c>
-      <c r="K8">
         <v>1.204</v>
       </c>
+      <c r="O8" t="s">
+        <v>5</v>
+      </c>
       <c r="P8" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q8" t="s">
-        <v>10</v>
-      </c>
-      <c r="R8" t="s">
         <v>51</v>
       </c>
-      <c r="S8" s="1" t="s">
+      <c r="R8" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="S8" t="s">
+        <v>7</v>
+      </c>
       <c r="T8" t="s">
-        <v>7</v>
-      </c>
-      <c r="U8" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>12</v>
       </c>
@@ -1102,37 +1083,34 @@
         <v>0</v>
       </c>
       <c r="H9">
-        <v>3</v>
+        <v>1000</v>
       </c>
       <c r="I9">
-        <v>1000</v>
+        <v>50</v>
       </c>
       <c r="J9">
-        <v>50</v>
-      </c>
-      <c r="K9">
         <v>1.016</v>
       </c>
+      <c r="O9" t="s">
+        <v>8</v>
+      </c>
       <c r="P9" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="Q9" t="s">
-        <v>12</v>
-      </c>
-      <c r="R9" t="s">
         <v>52</v>
       </c>
-      <c r="S9" s="1" t="s">
+      <c r="R9" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="S9" t="s">
+        <v>7</v>
+      </c>
       <c r="T9" t="s">
-        <v>7</v>
-      </c>
-      <c r="U9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>11</v>
       </c>
@@ -1146,37 +1124,34 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>1000</v>
       </c>
       <c r="I10">
-        <v>1000</v>
+        <v>50</v>
       </c>
       <c r="J10">
-        <v>50</v>
-      </c>
-      <c r="K10">
         <v>0.99850000000000005</v>
       </c>
+      <c r="O10" t="s">
+        <v>8</v>
+      </c>
       <c r="P10" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="Q10" t="s">
-        <v>11</v>
-      </c>
-      <c r="R10" t="s">
         <v>53</v>
       </c>
-      <c r="S10" s="1" t="s">
+      <c r="R10" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="S10" t="s">
+        <v>7</v>
+      </c>
       <c r="T10" t="s">
-        <v>7</v>
-      </c>
-      <c r="U10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>39</v>
       </c>
@@ -1186,73 +1161,70 @@
       <c r="G11" s="17">
         <v>97.330783938814534</v>
       </c>
+      <c r="O11" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="P11" s="1" t="s">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="S11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="T11" t="s">
+      <c r="S11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D12" t="s">
         <v>56</v>
       </c>
       <c r="G12" s="17">
         <v>35.496509410102867</v>
       </c>
-      <c r="N12" s="19">
-        <f>90.7*L3</f>
-        <v>1.0548409999999999</v>
+      <c r="M12" s="19"/>
+      <c r="O12" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="S12" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="T12" t="s">
+      <c r="S12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D13" t="s">
         <v>57</v>
       </c>
       <c r="G13" s="17">
         <v>46.935294117647068</v>
       </c>
+      <c r="O13" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="P13" s="1" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="S13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="T13" t="s">
+      <c r="S13" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>41</v>
       </c>
@@ -1262,69 +1234,69 @@
       <c r="G14" s="17">
         <v>0.36000000000000004</v>
       </c>
+      <c r="O14" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="P14" s="1" t="s">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="S14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="T14" t="s">
+      <c r="S14" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D15" t="s">
         <v>59</v>
       </c>
       <c r="G15" s="17">
         <v>0.36000000000000004</v>
       </c>
-      <c r="P15" s="1" t="s">
+      <c r="O15" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="P15" t="s">
+        <v>47</v>
+      </c>
       <c r="Q15" t="s">
-        <v>47</v>
-      </c>
-      <c r="R15" t="s">
         <v>48</v>
       </c>
-      <c r="S15" s="1" t="s">
+      <c r="R15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="T15" t="s">
+      <c r="S15" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D16" s="1" t="s">
         <v>60</v>
       </c>
       <c r="G16" s="17">
         <v>46.249920000000003</v>
       </c>
-      <c r="P16" s="1" t="s">
+      <c r="O16" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="P16" t="s">
+        <v>49</v>
+      </c>
       <c r="Q16" t="s">
-        <v>49</v>
-      </c>
-      <c r="R16" t="s">
         <v>65</v>
       </c>
-      <c r="S16" s="1" t="s">
+      <c r="R16" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="T16" t="s">
+      <c r="S16" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>43</v>
       </c>
@@ -1335,7 +1307,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>45</v>
       </c>
@@ -1346,7 +1318,7 @@
         <v>0.36000000000000004</v>
       </c>
     </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>47</v>
       </c>
@@ -1357,7 +1329,7 @@
         <v>0.36000000000000004</v>
       </c>
     </row>
-    <row r="20" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>49</v>
       </c>
@@ -1367,25 +1339,25 @@
       <c r="G20">
         <v>0.36000000000000004</v>
       </c>
-      <c r="K20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="L20" s="1"/>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
-      <c r="P20" s="1"/>
-    </row>
-    <row r="21" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="K21" s="1"/>
+    </row>
+    <row r="21" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="J21" s="1"/>
+      <c r="L21" s="1"/>
       <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="S21" s="8"/>
-    </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="K26" s="2"/>
-    </row>
-    <row r="27" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="K27" s="1"/>
+      <c r="R21" s="8"/>
+    </row>
+    <row r="26" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="J27" s="1"/>
+      <c r="L27" s="1"/>
       <c r="M27" s="1"/>
-      <c r="N27" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>